<commit_message>
Excel - LED strip update
</commit_message>
<xml_diff>
--- a/material.xlsx
+++ b/material.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VS\Projekty\AdvancedPianistRobot\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\janbe\Documents\VSB\AdvancedPianistRobot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7818ACC4-E9C4-4942-99E3-5E24F6929A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3968A020-0762-4173-BDD8-5C22926754AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="0" windowWidth="14400" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Název</t>
   </si>
@@ -49,16 +49,51 @@
   </si>
   <si>
     <t>LED pásky</t>
+  </si>
+  <si>
+    <t>Neon kryt pro LED</t>
+  </si>
+  <si>
+    <t>https://eshop.ledsolution.cz/silikonovy-neon-profil/?variantId=127930</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>https://pajenicko.cz/inteligentni-rgb-led-pasek-2m-ws2812-neopixel-100led-m-30w-m   https://www.digitalni-led.cz/product/digitalni-adresovatelne-led-pasky-ws2811/ws2812b-5v/led-pasek-digitalni-ws2812b_-5v_-100led_/58   https://www.digitalni-led.cz/product/cob-led-pasky/digital-cob-adresovatelne/digitalni-cob-led-pasek-ws2812b_-5v_-100/208</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005007982624217.html   https://www.aliexpress.com/item/1005006989400367.html</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005004792064706.html   https://www.aliexpress.com/item/4000966039097.html   https://www.aliexpress.com/item/4000077271746.html   https://www.aliexpress.com/item/1005005557329466.html</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -81,13 +116,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hypertextový odkaz" xfId="1" builtinId="8"/>
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -366,49 +405,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.21875" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="4" max="4" width="214.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
+      <c r="D6" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D6" r:id="rId1" display="https://www.aliexpress.com/item/1005007982624217.html   " xr:uid="{C94056BB-6133-4BC0-BFA7-33E8E648CD62}"/>
+    <hyperlink ref="D7" r:id="rId2" display="https://pajenicko.cz/inteligentni-rgb-led-pasek-2m-ws2812-neopixel-100led-m-30w-m   " xr:uid="{065C88C3-9E02-4BDB-A3F8-FA03C7D88553}"/>
+    <hyperlink ref="D9" r:id="rId3" xr:uid="{BE94E6CC-70B6-4FD9-A20D-3A105D12B070}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
RTOS folder + LEDs_klavesy code, materials.xlsx LEDs amount + prices, UCTENKY_FAKTURY folder + PNG receipts
</commit_message>
<xml_diff>
--- a/material.xlsx
+++ b/material.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\janbe\Documents\VSB\AdvancedPianistRobot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3968A020-0762-4173-BDD8-5C22926754AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7021EA85-BC2F-44FB-8014-F3FA3F836C61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>Název</t>
   </si>
@@ -33,9 +33,6 @@
     <t>Počet</t>
   </si>
   <si>
-    <t xml:space="preserve">Cena </t>
-  </si>
-  <si>
     <t>ethernet kabel</t>
   </si>
   <si>
@@ -54,25 +51,34 @@
     <t>Neon kryt pro LED</t>
   </si>
   <si>
-    <t>https://eshop.ledsolution.cz/silikonovy-neon-profil/?variantId=127930</t>
-  </si>
-  <si>
     <t>Link</t>
   </si>
   <si>
-    <t>https://pajenicko.cz/inteligentni-rgb-led-pasek-2m-ws2812-neopixel-100led-m-30w-m   https://www.digitalni-led.cz/product/digitalni-adresovatelne-led-pasky-ws2811/ws2812b-5v/led-pasek-digitalni-ws2812b_-5v_-100led_/58   https://www.digitalni-led.cz/product/cob-led-pasky/digital-cob-adresovatelne/digitalni-cob-led-pasek-ws2812b_-5v_-100/208</t>
-  </si>
-  <si>
-    <t>https://www.aliexpress.com/item/1005007982624217.html   https://www.aliexpress.com/item/1005006989400367.html</t>
-  </si>
-  <si>
-    <t>https://www.aliexpress.com/item/1005004792064706.html   https://www.aliexpress.com/item/4000966039097.html   https://www.aliexpress.com/item/4000077271746.html   https://www.aliexpress.com/item/1005005557329466.html</t>
+    <t>https://www.aliexpress.com/item/1005006989400367.html</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005007982624217.html</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005007705654602.html</t>
+  </si>
+  <si>
+    <t>2m</t>
+  </si>
+  <si>
+    <t>Cena</t>
+  </si>
+  <si>
+    <t>5m</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="#,##0.00\ &quot;Kč&quot;"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -120,10 +126,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hypertextový odkaz" xfId="1" builtinId="8"/>
@@ -409,7 +416,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" customWidth="1"/>
-    <col min="4" max="4" width="214.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" customWidth="1"/>
+    <col min="4" max="4" width="202.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -420,65 +428,83 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C3" s="3"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="C4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="3">
+        <v>177.96</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="3">
+        <v>192.25</v>
+      </c>
       <c r="D7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" t="s">
-        <v>13</v>
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="3">
+        <v>321.88</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D9" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="D9" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D6" r:id="rId1" display="https://www.aliexpress.com/item/1005007982624217.html   " xr:uid="{C94056BB-6133-4BC0-BFA7-33E8E648CD62}"/>
-    <hyperlink ref="D7" r:id="rId2" display="https://pajenicko.cz/inteligentni-rgb-led-pasek-2m-ws2812-neopixel-100led-m-30w-m   " xr:uid="{065C88C3-9E02-4BDB-A3F8-FA03C7D88553}"/>
-    <hyperlink ref="D9" r:id="rId3" xr:uid="{BE94E6CC-70B6-4FD9-A20D-3A105D12B070}"/>
+    <hyperlink ref="D8" r:id="rId1" xr:uid="{4BD92845-476D-426A-A759-9B5E48C057A0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lukii -> material update, api code, btnSongs now send api post request
</commit_message>
<xml_diff>
--- a/material.xlsx
+++ b/material.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Disk\Vysoka skola\Magisterske_studium\3_semester\Project_AdvancedPianistRobot\AdvancedPianistRobot\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VS\Projekty\AdvancedPianistRobot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{850EEB63-DC5B-469E-9BE0-AD2BF7F633F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A847D6-4AC1-4048-A217-32F012B9C720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-3060" windowWidth="38640" windowHeight="21390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
   <si>
     <t>Název</t>
   </si>
@@ -87,10 +87,49 @@
     <t>2ks (2m)</t>
   </si>
   <si>
-    <t>Od Slaniny</t>
-  </si>
-  <si>
     <t>-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stepdown měnič </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLA filament </t>
+  </si>
+  <si>
+    <t>https://www.hadex.cz/m411a-napajeci-modul-step-down-menic-6-40v15-35v-20a/</t>
+  </si>
+  <si>
+    <t>2 ks</t>
+  </si>
+  <si>
+    <t>1 ks</t>
+  </si>
+  <si>
+    <t>https://www.prusa3d.com/cs/produkt/prusament-pla-jet-black-2kg/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dutinky </t>
+  </si>
+  <si>
+    <t>https://www.hadex.cz/l839e-sada-dutinek-izolovanych-05-6mm2-celkem-800ks/</t>
+  </si>
+  <si>
+    <t>https://www.hadex.cz/d454a-sm-dupont-konektory-2-4pin-s-rozteci-254mm-sada-480ks/</t>
+  </si>
+  <si>
+    <t>SM dupont konektory</t>
+  </si>
+  <si>
+    <t>https://www.hadex.cz/n126-dvojlinka-2x15mm2-cu16awg-cerveno-cerna-cyh-2x15mm/</t>
+  </si>
+  <si>
+    <t>Dvojlinka 2x1,5mm2</t>
+  </si>
+  <si>
+    <t>5 m</t>
+  </si>
+  <si>
+    <t>Dostaneme od doc. Ing. Zdeněk Slanina, Ph.D.</t>
   </si>
 </sst>
 </file>
@@ -434,15 +473,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" customWidth="1"/>
-    <col min="4" max="4" width="202.28515625" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" customWidth="1"/>
+    <col min="4" max="4" width="202.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -456,21 +495,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -480,39 +519,39 @@
       <c r="C3" s="3">
         <v>469</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -526,7 +565,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>14</v>
       </c>
@@ -537,7 +576,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -551,7 +590,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -563,13 +602,89 @@
       </c>
       <c r="D9" s="1" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="3">
+        <v>215</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="3">
+        <v>1300</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="3">
+        <v>245</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="3">
+        <v>195</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="3">
+        <v>26</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D8" r:id="rId1" xr:uid="{4BD92845-476D-426A-A759-9B5E48C057A0}"/>
+    <hyperlink ref="D12" r:id="rId2" xr:uid="{E7F642ED-F160-4CB7-B276-67D6A6B86841}"/>
+    <hyperlink ref="D10" r:id="rId3" xr:uid="{C0D1450B-EDC4-4545-944E-0469ADAA31F1}"/>
+    <hyperlink ref="D11" r:id="rId4" xr:uid="{8DF5CD03-5C59-4179-A9B9-D772F970D7C8}"/>
+    <hyperlink ref="D13" r:id="rId5" xr:uid="{F114B684-C4B8-4D76-B235-07BB59913D97}"/>
+    <hyperlink ref="D3" r:id="rId6" xr:uid="{5DA90DCE-D24D-49C0-9D6F-3B84F658D6C2}"/>
+    <hyperlink ref="D14" r:id="rId7" xr:uid="{726C3A6D-3F0B-4CEA-AE07-6CCEF00F5E5F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>